<commit_message>
Stage 8 review fixes: C-024
</commit_message>
<xml_diff>
--- a/output/archive/Archive/Users/mrinalvesi_old_laptop/DMPK/Working/Accession_Handover_052019_v3.xlsx
+++ b/output/archive/Archive/Users/mrinalvesi_old_laptop/DMPK/Working/Accession_Handover_052019_v3.xlsx
@@ -162,9 +162,9 @@
     <author>Megan Larkin</author>
   </authors>
   <commentList>
-    <comment ref="C6" authorId="0" shapeId="0">
+    <comment ref="C7" authorId="0" shapeId="0">
       <text>
-        <t>Check whether the SC- prefix is still on the older paper log</t>
+        <t>Check the older paper log before treating an informal prefix as a LIMS accession.</t>
       </text>
     </comment>
   </commentList>
@@ -750,17 +750,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>SC-</t>
+          <t>Local scratch tracking</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Scratch sample tracking, not for client files</t>
+          <t>Consult the older sample log for any informal prefixes</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not for client files</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Accession and project numbers stay as they are when the group naming starts.</t>
+          <t>Use the original accession and project identifiers when retrieving archived records.</t>
         </is>
       </c>
     </row>
@@ -825,12 +825,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Client_Work/&lt;project&gt;/Memos</t>
+          <t>Client_Work study folder</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Scan of the signed copy kept with the PDF</t>
+          <t>Check the study file index for the signed copy</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Archive/Users/Working/Memos</t>
+          <t>Personal DMPK working folder</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Client_Work/&lt;project&gt;/QC</t>
+          <t>Study records linked to the assay worksheet</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Stored with the assay worksheet</t>
+          <t>Use the study index for the archived location</t>
         </is>
       </c>
     </row>
@@ -876,12 +876,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Filing room, shelf 3</t>
+          <t>Paper archive; consult the archive note</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Incomplete. See the archive note.</t>
+          <t>Incomplete.</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Several links in the 2017 memos point at folders that have since moved.</t>
+          <t>Working location notes: verify the study index before using an old memo link.</t>
         </is>
       </c>
     </row>

</xml_diff>